<commit_message>
fix(xlsx): preserve threaded comment metadata through edits
</commit_message>
<xml_diff>
--- a/src/core/xlsx/__fixtures__/excel-threaded-comments.xlsx
+++ b/src/core/xlsx/__fixtures__/excel-threaded-comments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Development\ooxml-parity-x14\src\core\xlsx\__fixtures__\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB446935-E273-4975-A26D-70EA179367C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5DCFE10-2796-4F03-8A4D-0DC371F52B56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{6FC71AA2-ABEC-4C25-A665-BB311EFC8D71}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{44282300-07F2-4AEF-A822-823249E4DD14}"/>
   </bookViews>
   <sheets>
     <sheet name="Comments" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={41A480B0-6A22-40EA-A061-DBCF0D5BD85B}</author>
+    <author>tc={1A8EEA06-0338-4DD5-8751-5E280CA57A59}</author>
   </authors>
   <commentList>
-    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{41A480B0-6A22-40EA-A061-DBCF0D5BD85B}">
+    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{1A8EEA06-0338-4DD5-8751-5E280CA57A59}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -55,6 +55,14 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+  <si>
+    <t>Threaded comment cell</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -115,7 +123,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Parity Author" id="{A8147C65-A90A-44AC-8620-CFA6A9A56374}" userId="Parity Author" providerId="None"/>
+  <person displayName="Parity Author" id="{AAAAAAAA-0000-4000-8000-000000000001}" userId="Parity Author" providerId="None"/>
 </personList>
 </file>
 
@@ -436,24 +444,28 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B2" dT="2026-10-31T00:01:03.38" personId="{A8147C65-A90A-44AC-8620-CFA6A9A56374}" id="{41A480B0-6A22-40EA-A061-DBCF0D5BD85B}">
+  <threadedComment ref="B2" dT="2026-10-31T01:03:29.98" personId="{AAAAAAAA-0000-4000-8000-000000000001}" id="{1A8EEA06-0338-4DD5-8751-5E280CA57A59}">
     <text>Original comment</text>
   </threadedComment>
-  <threadedComment ref="B2" dT="2026-10-31T00:01:03.59" personId="{A8147C65-A90A-44AC-8620-CFA6A9A56374}" id="{D5957A65-4336-40D9-87EE-2DD16CAA499A}" parentId="{41A480B0-6A22-40EA-A061-DBCF0D5BD85B}">
+  <threadedComment ref="B2" dT="2026-10-31T01:03:30.02" personId="{AAAAAAAA-0000-4000-8000-000000000001}" id="{8CD1615D-480E-409C-B6E9-AB1B7672A25A}" parentId="{1A8EEA06-0338-4DD5-8751-5E280CA57A59}">
     <text>First reply</text>
   </threadedComment>
-  <threadedComment ref="B2" dT="2026-10-31T00:01:03.59" personId="{A8147C65-A90A-44AC-8620-CFA6A9A56374}" id="{D5957A65-4336-40DA-87EE-2DD16CAA499A}" parentId="{41A480B0-6A22-40EA-A061-DBCF0D5BD85B}">
+  <threadedComment ref="B2" dT="2026-10-31T01:03:30.02" personId="{AAAAAAAA-0000-4000-8000-000000000001}" id="{8CD1615D-480E-409D-B6E9-AB1B7672A25A}" parentId="{1A8EEA06-0338-4DD5-8751-5E280CA57A59}">
     <text>Second reply</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C728E284-A953-459C-BF4D-0E6AA0313C45}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3C7AD289-2D6A-4CC9-834E-41FBE789E5D4}">
   <dimension ref="B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>